<commit_message>
Adjust citation identification method
</commit_message>
<xml_diff>
--- a/examples/graph.node.xlsx
+++ b/examples/graph.node.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="97">
   <si>
     <t>doc_index</t>
   </si>
@@ -40,6 +40,12 @@
     <t>GCS</t>
   </si>
   <si>
+    <t>Iyer R</t>
+  </si>
+  <si>
+    <t>Iyer RM</t>
+  </si>
+  <si>
     <t>Iver R</t>
   </si>
   <si>
@@ -49,76 +55,154 @@
     <t>Byrne W</t>
   </si>
   <si>
+    <t>Chen SF</t>
+  </si>
+  <si>
     <t>Schwenk H</t>
   </si>
   <si>
     <t>Bengio Y</t>
   </si>
   <si>
+    <t>Kwon OW</t>
+  </si>
+  <si>
     <t>Castro MJ</t>
   </si>
   <si>
+    <t>Whittaker EWD</t>
+  </si>
+  <si>
+    <t>Fang GL</t>
+  </si>
+  <si>
+    <t>Emami A</t>
+  </si>
+  <si>
+    <t>Arisoy E</t>
+  </si>
+  <si>
+    <t>Wang C</t>
+  </si>
+  <si>
     <t>Kirchhoff K</t>
   </si>
   <si>
+    <t>Choueiter G</t>
+  </si>
+  <si>
     <t>Hirsimaki T</t>
   </si>
   <si>
-    <t>Tur G</t>
+    <t>Alumae T</t>
+  </si>
+  <si>
+    <t>Huang S</t>
+  </si>
+  <si>
+    <t>Rotovnik T</t>
+  </si>
+  <si>
+    <t>Xu P</t>
+  </si>
+  <si>
+    <t>Roark B</t>
+  </si>
+  <si>
+    <t>Zitouni I</t>
   </si>
   <si>
     <t>Siivola V</t>
   </si>
   <si>
+    <t>Sarikaya R</t>
+  </si>
+  <si>
+    <t>Ke J</t>
+  </si>
+  <si>
+    <t>Xu PY</t>
+  </si>
+  <si>
+    <t>Sethy A</t>
+  </si>
+  <si>
+    <t>Wichmann S</t>
+  </si>
+  <si>
+    <t>Huang SF</t>
+  </si>
+  <si>
     <t>Deoras A</t>
   </si>
   <si>
-    <t>Arisoy E</t>
-  </si>
-  <si>
-    <t>Haznedaroglu A</t>
+    <t>Kurata G</t>
+  </si>
+  <si>
+    <t>Nettle D</t>
+  </si>
+  <si>
+    <t>Chen B</t>
   </si>
   <si>
     <t>Sundermeyer M</t>
   </si>
   <si>
-    <t>Liu X</t>
-  </si>
-  <si>
     <t>Chen X</t>
   </si>
   <si>
     <t>Botha JA</t>
   </si>
   <si>
+    <t>Koller O</t>
+  </si>
+  <si>
+    <t>Brychcin T</t>
+  </si>
+  <si>
+    <t>Nguyen AT</t>
+  </si>
+  <si>
+    <t>Liu XY</t>
+  </si>
+  <si>
+    <t>Varjokallio M</t>
+  </si>
+  <si>
+    <t>Irie K</t>
+  </si>
+  <si>
+    <t>Gangireddy SR</t>
+  </si>
+  <si>
     <t>Kurimo M</t>
   </si>
   <si>
-    <t>Grave E</t>
+    <t>Ma M</t>
   </si>
   <si>
     <t>Enarvi S</t>
   </si>
   <si>
-    <t>Dauphin YN</t>
-  </si>
-  <si>
-    <t>Wang DL</t>
-  </si>
-  <si>
-    <t>Yang Q</t>
-  </si>
-  <si>
-    <t>Al-Rfou R</t>
-  </si>
-  <si>
-    <t>Guu K</t>
-  </si>
-  <si>
-    <t>Li ZH</t>
-  </si>
-  <si>
-    <t>Zhu H</t>
+    <t>Hellendoorn VJ</t>
+  </si>
+  <si>
+    <t>Huang J</t>
+  </si>
+  <si>
+    <t>Nguyen S</t>
+  </si>
+  <si>
+    <t>Sridhar A</t>
+  </si>
+  <si>
+    <t>Sincan OM</t>
+  </si>
+  <si>
+    <t>IEEE SIGNAL PROCESSING LETTERS</t>
+  </si>
+  <si>
+    <t>IEEE TRANSACTIONS ON SPEECH AND AUDIO PROCESSING</t>
   </si>
   <si>
     <t>COMPUTER SPEECH AND LANGUAGE</t>
@@ -136,58 +220,91 @@
     <t>JOURNAL OF MACHINE LEARNING RESEARCH</t>
   </si>
   <si>
+    <t>SPEECH COMMUNICATION</t>
+  </si>
+  <si>
     <t>COMPUTATIONAL METHODS IN NEURAL MODELING, PT 1</t>
   </si>
   <si>
     <t>2004 IEEE INTERNATIONAL JOINT CONFERENCE ON NEURAL NETWORKS, VOLS 1-4, PROCEEDINGS</t>
   </si>
   <si>
-    <t>2007 IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS, SPEECH, AND SIGNAL PROCESSING, VOL IV, PTS 1-3</t>
+    <t>IEEE TRANSACTIONS ON SYSTEMS MAN AND CYBERNETICS PART A-SYSTEMS AND HUMANS</t>
+  </si>
+  <si>
+    <t>MACHINE LEARNING</t>
+  </si>
+  <si>
+    <t>SIGNAL PROCESSING</t>
+  </si>
+  <si>
+    <t>LANGUAGE RESOURCES AND EVALUATION</t>
+  </si>
+  <si>
+    <t>2006 IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS, SPEECH AND SIGNAL PROCESSING, VOLS 1-13</t>
+  </si>
+  <si>
+    <t>2007 IEEE WORKSHOP ON AUTOMATIC SPEECH RECOGNITION AND UNDERSTANDING, VOLS 1 AND 2</t>
   </si>
   <si>
     <t>IEEE TRANSACTIONS ON AUDIO SPEECH AND LANGUAGE PROCESSING</t>
   </si>
   <si>
+    <t>COMMUNICATIONS IN COMPUTATIONAL PHYSICS</t>
+  </si>
+  <si>
+    <t>2009 IEEE WORKSHOP ON AUTOMATIC SPEECH RECOGNITION &amp; UNDERSTANDING (ASRU 2009)</t>
+  </si>
+  <si>
+    <t>HUMAN BIOLOGY</t>
+  </si>
+  <si>
     <t>2011 IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS, SPEECH, AND SIGNAL PROCESSING</t>
   </si>
   <si>
-    <t>SPEECH COMMUNICATION</t>
+    <t>PHILOSOPHICAL TRANSACTIONS OF THE ROYAL SOCIETY B-BIOLOGICAL SCIENCES</t>
+  </si>
+  <si>
+    <t>INFORMATION PROCESSING &amp; MANAGEMENT</t>
   </si>
   <si>
     <t>IEEE-ACM TRANSACTIONS ON AUDIO SPEECH AND LANGUAGE PROCESSING</t>
   </si>
   <si>
-    <t>2014 IEEE INTERNATIONAL CONFERENCE ON ACOUSTICS, SPEECH AND SIGNAL PROCESSING (ICASSP)</t>
-  </si>
-  <si>
     <t>15TH ANNUAL CONFERENCE OF THE INTERNATIONAL SPEECH COMMUNICATION ASSOCIATION (INTERSPEECH 2014), VOLS 1-4</t>
   </si>
   <si>
     <t>INTERNATIONAL CONFERENCE ON MACHINE LEARNING, VOL 32 (CYCLE 2)</t>
   </si>
   <si>
-    <t>LANGUAGE RESOURCES AND EVALUATION</t>
-  </si>
-  <si>
-    <t>ADVANCES IN NEURAL INFORMATION PROCESSING SYSTEMS 30 (NIPS 2017)</t>
-  </si>
-  <si>
-    <t>INTERNATIONAL CONFERENCE ON MACHINE LEARNING, VOL 70</t>
-  </si>
-  <si>
-    <t>INTERNATIONAL CONFERENCE ON MACHINE LEARNING, VOL 97</t>
-  </si>
-  <si>
-    <t>ADVANCES IN NEURAL INFORMATION PROCESSING SYSTEMS 32 (NIPS 2019)</t>
-  </si>
-  <si>
-    <t>THIRTY-THIRD AAAI CONFERENCE ON ARTIFICIAL INTELLIGENCE / THIRTY-FIRST INNOVATIVE APPLICATIONS OF ARTIFICIAL INTELLIGENCE CONFERENCE / NINTH AAAI SYMPOSIUM ON EDUCATIONAL ADVANCES IN ARTIFICIAL INTELLIGENCE</t>
-  </si>
-  <si>
-    <t>INTERNATIONAL CONFERENCE ON MACHINE LEARNING, VOL 119</t>
-  </si>
-  <si>
-    <t>INTERNATIONAL CONFERENCE ON MACHINE LEARNING, VOL 139</t>
+    <t>COMPUTER VISION AND IMAGE UNDERSTANDING</t>
+  </si>
+  <si>
+    <t>2015 IEEE/ACM 37TH IEEE INTERNATIONAL CONFERENCE ON SOFTWARE ENGINEERING, VOL 1</t>
+  </si>
+  <si>
+    <t>STATISTICAL LANGUAGE AND SPEECH PROCESSING, SLSP 2016</t>
+  </si>
+  <si>
+    <t>17TH ANNUAL CONFERENCE OF THE INTERNATIONAL SPEECH COMMUNICATION ASSOCIATION (INTERSPEECH 2016), VOLS 1-5: UNDERSTANDING SPEECH PROCESSING IN HUMANS AND MACHINES</t>
+  </si>
+  <si>
+    <t>18TH ANNUAL CONFERENCE OF THE INTERNATIONAL SPEECH COMMUNICATION ASSOCIATION (INTERSPEECH 2017), VOLS 1-6: SITUATED INTERACTION</t>
+  </si>
+  <si>
+    <t>ESEC/FSE 2017: PROCEEDINGS OF THE 2017 11TH JOINT MEETING ON FOUNDATIONS OF SOFTWARE ENGINEERING</t>
+  </si>
+  <si>
+    <t>IEEE TRANSACTIONS ON CIRCUITS AND SYSTEMS FOR VIDEO TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>34TH IEEE/ACM INTERNATIONAL CONFERENCE ON AUTOMATED SOFTWARE ENGINEERING (ASE 2019)</t>
+  </si>
+  <si>
+    <t>MM '20: PROCEEDINGS OF THE 28TH ACM INTERNATIONAL CONFERENCE ON MULTIMEDIA</t>
+  </si>
+  <si>
+    <t>IEEE ACCESS</t>
   </si>
 </sst>
 </file>
@@ -545,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -576,486 +693,507 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2">
-        <v>1999</v>
+        <v>1997</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E2">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>267</v>
+        <v>221</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H2">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
       <c r="C3">
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="E3">
-        <v>88</v>
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>1279</v>
+        <v>30</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H3">
-        <v>210</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
       <c r="C4">
-        <v>2000</v>
+        <v>1999</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>63</v>
+      </c>
+      <c r="E4">
+        <v>13</v>
       </c>
       <c r="F4">
-        <v>1029</v>
+        <v>267</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H4">
-        <v>40</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5">
-        <v>120</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5">
-        <v>2002</v>
+        <v>2000</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>62</v>
+      </c>
+      <c r="E5">
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>765</v>
+        <v>76</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
-        <v>135</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6">
-        <v>2003</v>
+        <v>2000</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>88</v>
       </c>
       <c r="F6">
-        <v>1137</v>
+        <v>1279</v>
       </c>
       <c r="G6">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>1873</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7">
-        <v>144</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7">
-        <v>2003</v>
+        <v>2000</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7">
-        <v>2686</v>
+        <v>65</v>
       </c>
       <c r="F7">
-        <v>598</v>
+        <v>1029</v>
       </c>
       <c r="G7">
         <v>3</v>
       </c>
       <c r="H7">
-        <v>9</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8">
-        <v>161</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C8">
-        <v>2004</v>
+        <v>2000</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>62</v>
+      </c>
+      <c r="E8">
+        <v>8</v>
       </c>
       <c r="F8">
-        <v>3059</v>
+        <v>37</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H8">
-        <v>13</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="C9">
-        <v>2006</v>
+        <v>2002</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="F9">
-        <v>589</v>
+        <v>765</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>61</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10">
-        <v>253</v>
+        <v>135</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
       </c>
       <c r="C10">
-        <v>2006</v>
+        <v>2003</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="E10">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="F10">
-        <v>515</v>
+        <v>1137</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>73</v>
       </c>
       <c r="H10">
-        <v>66</v>
+        <v>1873</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11">
-        <v>273</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C11">
-        <v>2007</v>
+        <v>2003</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="E11">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="F11">
-        <v>492</v>
+        <v>287</v>
       </c>
       <c r="G11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="H11">
-        <v>249</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12">
-        <v>276</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12">
-        <v>2007</v>
+        <v>2003</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>69</v>
+      </c>
+      <c r="E12">
+        <v>2686</v>
       </c>
       <c r="F12">
-        <v>173</v>
+        <v>598</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13">
-        <v>301</v>
+        <v>149</v>
       </c>
       <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13">
+        <v>2003</v>
+      </c>
+      <c r="D13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13">
         <v>17</v>
       </c>
-      <c r="C13">
-        <v>2007</v>
-      </c>
-      <c r="D13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13">
-        <v>15</v>
-      </c>
       <c r="F13">
-        <v>1617</v>
+        <v>87</v>
       </c>
       <c r="G13">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H13">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14">
-        <v>502</v>
+        <v>161</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C14">
-        <v>2011</v>
+        <v>2004</v>
       </c>
       <c r="D14" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="F14">
-        <v>5532</v>
+        <v>3059</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15">
-        <v>609</v>
+        <v>165</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15">
-        <v>2013</v>
+        <v>2004</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="E15">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="F15">
-        <v>162</v>
+        <v>305</v>
       </c>
       <c r="G15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>22</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16">
-        <v>645</v>
+        <v>193</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16">
-        <v>2014</v>
+        <v>2005</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="E16">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="F16">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17">
-        <v>648</v>
+        <v>219</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17">
-        <v>2014</v>
+        <v>2006</v>
       </c>
       <c r="D17" t="s">
-        <v>47</v>
+        <v>73</v>
+      </c>
+      <c r="E17">
+        <v>86</v>
+      </c>
+      <c r="F17">
+        <v>2844</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18">
-        <v>662</v>
+        <v>236</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18">
-        <v>2014</v>
+        <v>2006</v>
       </c>
       <c r="D18" t="s">
-        <v>48</v>
+        <v>74</v>
+      </c>
+      <c r="E18">
+        <v>40</v>
       </c>
       <c r="F18">
-        <v>661</v>
+        <v>25</v>
       </c>
       <c r="G18">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19">
-        <v>668</v>
+        <v>240</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C19">
-        <v>2014</v>
+        <v>2006</v>
       </c>
       <c r="D19" t="s">
-        <v>47</v>
+        <v>63</v>
+      </c>
+      <c r="E19">
+        <v>20</v>
+      </c>
+      <c r="F19">
+        <v>589</v>
       </c>
       <c r="G19">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20">
-        <v>670</v>
+        <v>245</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C20">
-        <v>2014</v>
+        <v>2006</v>
       </c>
       <c r="D20" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="F20">
-        <v>641</v>
+        <v>1053</v>
       </c>
       <c r="G20">
         <v>4</v>
       </c>
       <c r="H20">
-        <v>27</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21">
-        <v>708</v>
+        <v>253</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C21">
-        <v>2014</v>
+        <v>2006</v>
       </c>
       <c r="D21" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="E21">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F21">
-        <v>1899</v>
+        <v>515</v>
       </c>
       <c r="G21">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H21">
         <v>66</v>
@@ -1063,290 +1201,1078 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22">
-        <v>749</v>
+        <v>254</v>
       </c>
       <c r="B22" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C22">
-        <v>2015</v>
+        <v>2006</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
-      </c>
-      <c r="E22">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="F22">
-        <v>517</v>
+        <v>429</v>
       </c>
       <c r="G22">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>296</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23">
-        <v>875</v>
+        <v>265</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C23">
-        <v>2016</v>
+        <v>2007</v>
       </c>
       <c r="D23" t="s">
-        <v>46</v>
+        <v>71</v>
       </c>
       <c r="E23">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F23">
-        <v>2146</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23">
-        <v>37</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24">
-        <v>915</v>
+        <v>272</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C24">
-        <v>2017</v>
+        <v>2007</v>
       </c>
       <c r="D24" t="s">
-        <v>50</v>
-      </c>
-      <c r="E24">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="F24">
-        <v>961</v>
+        <v>124</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25">
-        <v>970</v>
+        <v>273</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="C25">
-        <v>2017</v>
+        <v>2007</v>
       </c>
       <c r="D25" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="E25">
-        <v>30</v>
+        <v>21</v>
+      </c>
+      <c r="F25">
+        <v>492</v>
       </c>
       <c r="G25">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="H25">
-        <v>6</v>
+        <v>249</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26">
-        <v>975</v>
+        <v>275</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C26">
-        <v>2017</v>
+        <v>2007</v>
       </c>
       <c r="D26" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="E26">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F26">
-        <v>2085</v>
+        <v>437</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H26">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27">
-        <v>977</v>
+        <v>287</v>
       </c>
       <c r="B27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C27">
-        <v>2017</v>
+        <v>2007</v>
       </c>
       <c r="D27" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E27">
-        <v>70</v>
+        <v>21</v>
+      </c>
+      <c r="F27">
+        <v>105</v>
       </c>
       <c r="G27">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="H27">
-        <v>743</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28">
-        <v>1217</v>
+        <v>288</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C28">
-        <v>2019</v>
+        <v>2007</v>
       </c>
       <c r="D28" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="E28">
-        <v>97</v>
+        <v>21</v>
+      </c>
+      <c r="F28">
+        <v>373</v>
       </c>
       <c r="G28">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="H28">
-        <v>17</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29">
-        <v>1225</v>
+        <v>297</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C29">
-        <v>2019</v>
+        <v>2007</v>
       </c>
       <c r="D29" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E29">
-        <v>32</v>
+        <v>21</v>
+      </c>
+      <c r="F29">
+        <v>88</v>
       </c>
       <c r="G29">
-        <v>79</v>
+        <v>3</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30">
-        <v>1263</v>
+        <v>301</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C30">
-        <v>2019</v>
+        <v>2007</v>
       </c>
       <c r="D30" t="s">
-        <v>55</v>
+        <v>77</v>
+      </c>
+      <c r="E30">
+        <v>15</v>
       </c>
       <c r="F30">
-        <v>3159</v>
+        <v>1617</v>
       </c>
       <c r="G30">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H30">
-        <v>96</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31">
-        <v>1360</v>
+        <v>317</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C31">
-        <v>2020</v>
+        <v>2008</v>
       </c>
       <c r="D31" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="E31">
-        <v>119</v>
+        <v>16</v>
+      </c>
+      <c r="F31">
+        <v>1330</v>
       </c>
       <c r="G31">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="H31">
-        <v>122</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32">
-        <v>1471</v>
+        <v>325</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C32">
-        <v>2021</v>
+        <v>2008</v>
       </c>
       <c r="D32" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="E32">
-        <v>139</v>
+        <v>3</v>
+      </c>
+      <c r="F32">
+        <v>935</v>
       </c>
       <c r="G32">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33">
-        <v>1568</v>
+        <v>381</v>
       </c>
       <c r="B33" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="C33">
-        <v>2021</v>
+        <v>2009</v>
       </c>
       <c r="D33" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33">
+        <v>17</v>
+      </c>
+      <c r="F33">
+        <v>724</v>
+      </c>
+      <c r="G33">
+        <v>7</v>
+      </c>
+      <c r="H33">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34">
+        <v>389</v>
+      </c>
+      <c r="B34" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34">
+        <v>2009</v>
+      </c>
+      <c r="D34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F34">
+        <v>299</v>
+      </c>
+      <c r="G34">
+        <v>3</v>
+      </c>
+      <c r="H34">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35">
+        <v>391</v>
+      </c>
+      <c r="B35" t="s">
+        <v>35</v>
+      </c>
+      <c r="C35">
+        <v>2009</v>
+      </c>
+      <c r="D35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F35">
+        <v>317</v>
+      </c>
+      <c r="G35">
+        <v>5</v>
+      </c>
+      <c r="H35">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36">
+        <v>396</v>
+      </c>
+      <c r="B36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C36">
+        <v>2009</v>
+      </c>
+      <c r="D36" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36">
+        <v>17</v>
+      </c>
+      <c r="F36">
+        <v>13</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+      <c r="H36">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37">
+        <v>410</v>
+      </c>
+      <c r="B37" t="s">
+        <v>37</v>
+      </c>
+      <c r="C37">
+        <v>2009</v>
+      </c>
+      <c r="D37" t="s">
+        <v>80</v>
+      </c>
+      <c r="E37">
+        <v>81</v>
+      </c>
+      <c r="F37">
+        <v>259</v>
+      </c>
+      <c r="G37">
+        <v>3</v>
+      </c>
+      <c r="H37">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38">
+        <v>429</v>
+      </c>
+      <c r="B38" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38">
+        <v>2010</v>
+      </c>
+      <c r="D38" t="s">
+        <v>77</v>
+      </c>
+      <c r="E38">
+        <v>18</v>
+      </c>
+      <c r="F38">
+        <v>1941</v>
+      </c>
+      <c r="G38">
+        <v>2</v>
+      </c>
+      <c r="H38">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39">
+        <v>502</v>
+      </c>
+      <c r="B39" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39">
+        <v>2011</v>
+      </c>
+      <c r="D39" t="s">
+        <v>81</v>
+      </c>
+      <c r="F39">
+        <v>5532</v>
+      </c>
+      <c r="G39">
+        <v>10</v>
+      </c>
+      <c r="H39">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40">
+        <v>541</v>
+      </c>
+      <c r="B40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40">
+        <v>2012</v>
+      </c>
+      <c r="D40" t="s">
+        <v>68</v>
+      </c>
+      <c r="E40">
+        <v>54</v>
+      </c>
+      <c r="F40">
+        <v>219</v>
+      </c>
+      <c r="G40">
+        <v>3</v>
+      </c>
+      <c r="H40">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41">
+        <v>576</v>
+      </c>
+      <c r="B41" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41">
+        <v>2012</v>
+      </c>
+      <c r="D41" t="s">
+        <v>82</v>
+      </c>
+      <c r="E41">
+        <v>367</v>
+      </c>
+      <c r="F41">
+        <v>1829</v>
+      </c>
+      <c r="G41">
+        <v>3</v>
+      </c>
+      <c r="H41">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42">
+        <v>597</v>
+      </c>
+      <c r="B42" t="s">
+        <v>42</v>
+      </c>
+      <c r="C42">
+        <v>2013</v>
+      </c>
+      <c r="D42" t="s">
+        <v>83</v>
+      </c>
+      <c r="E42">
+        <v>49</v>
+      </c>
+      <c r="F42">
+        <v>807</v>
+      </c>
+      <c r="G42">
+        <v>4</v>
+      </c>
+      <c r="H42">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43">
+        <v>609</v>
+      </c>
+      <c r="B43" t="s">
+        <v>39</v>
+      </c>
+      <c r="C43">
+        <v>2013</v>
+      </c>
+      <c r="D43" t="s">
+        <v>68</v>
+      </c>
+      <c r="E43">
+        <v>55</v>
+      </c>
+      <c r="F43">
+        <v>162</v>
+      </c>
+      <c r="G43">
+        <v>8</v>
+      </c>
+      <c r="H43">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44">
+        <v>645</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44">
+        <v>2014</v>
+      </c>
+      <c r="D44" t="s">
+        <v>84</v>
+      </c>
+      <c r="E44">
+        <v>22</v>
+      </c>
+      <c r="F44">
+        <v>184</v>
+      </c>
+      <c r="G44">
+        <v>5</v>
+      </c>
+      <c r="H44">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45">
+        <v>662</v>
+      </c>
+      <c r="B45" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45">
+        <v>2014</v>
+      </c>
+      <c r="D45" t="s">
+        <v>85</v>
+      </c>
+      <c r="F45">
+        <v>661</v>
+      </c>
+      <c r="G45">
+        <v>11</v>
+      </c>
+      <c r="H45">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46">
+        <v>670</v>
+      </c>
+      <c r="B46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C46">
+        <v>2014</v>
+      </c>
+      <c r="D46" t="s">
+        <v>85</v>
+      </c>
+      <c r="F46">
+        <v>641</v>
+      </c>
+      <c r="G46">
+        <v>4</v>
+      </c>
+      <c r="H46">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47">
+        <v>708</v>
+      </c>
+      <c r="B47" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47">
+        <v>2014</v>
+      </c>
+      <c r="D47" t="s">
+        <v>86</v>
+      </c>
+      <c r="E47">
+        <v>32</v>
+      </c>
+      <c r="F47">
+        <v>1899</v>
+      </c>
+      <c r="G47">
+        <v>4</v>
+      </c>
+      <c r="H47">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48">
+        <v>737</v>
+      </c>
+      <c r="B48" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48">
+        <v>2015</v>
+      </c>
+      <c r="D48" t="s">
+        <v>87</v>
+      </c>
+      <c r="E48">
+        <v>141</v>
+      </c>
+      <c r="F48">
+        <v>108</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49">
+        <v>739</v>
+      </c>
+      <c r="B49" t="s">
+        <v>47</v>
+      </c>
+      <c r="C49">
+        <v>2015</v>
+      </c>
+      <c r="D49" t="s">
+        <v>63</v>
+      </c>
+      <c r="E49">
+        <v>33</v>
+      </c>
+      <c r="F49">
+        <v>88</v>
+      </c>
+      <c r="G49">
+        <v>3</v>
+      </c>
+      <c r="H49">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50">
+        <v>749</v>
+      </c>
+      <c r="B50" t="s">
+        <v>43</v>
+      </c>
+      <c r="C50">
+        <v>2015</v>
+      </c>
+      <c r="D50" t="s">
+        <v>84</v>
+      </c>
+      <c r="E50">
+        <v>23</v>
+      </c>
+      <c r="F50">
+        <v>517</v>
+      </c>
+      <c r="G50">
+        <v>16</v>
+      </c>
+      <c r="H50">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51">
+        <v>793</v>
+      </c>
+      <c r="B51" t="s">
+        <v>48</v>
+      </c>
+      <c r="C51">
+        <v>2015</v>
+      </c>
+      <c r="D51" t="s">
+        <v>88</v>
+      </c>
+      <c r="F51">
+        <v>858</v>
+      </c>
+      <c r="G51">
+        <v>4</v>
+      </c>
+      <c r="H51">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52">
+        <v>821</v>
+      </c>
+      <c r="B52" t="s">
+        <v>49</v>
+      </c>
+      <c r="C52">
+        <v>2016</v>
+      </c>
+      <c r="D52" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52">
+        <v>24</v>
+      </c>
+      <c r="F52">
+        <v>1438</v>
+      </c>
+      <c r="G52">
+        <v>6</v>
+      </c>
+      <c r="H52">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53">
+        <v>827</v>
+      </c>
+      <c r="B53" t="s">
+        <v>50</v>
+      </c>
+      <c r="C53">
+        <v>2016</v>
+      </c>
+      <c r="D53" t="s">
+        <v>89</v>
+      </c>
+      <c r="E53">
+        <v>9918</v>
+      </c>
+      <c r="F53">
+        <v>133</v>
+      </c>
+      <c r="G53">
+        <v>3</v>
+      </c>
+      <c r="H53">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54">
+        <v>859</v>
+      </c>
+      <c r="B54" t="s">
+        <v>51</v>
+      </c>
+      <c r="C54">
+        <v>2016</v>
+      </c>
+      <c r="D54" t="s">
+        <v>90</v>
+      </c>
+      <c r="F54">
+        <v>3519</v>
+      </c>
+      <c r="G54">
+        <v>3</v>
+      </c>
+      <c r="H54">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55">
+        <v>875</v>
+      </c>
+      <c r="B55" t="s">
+        <v>44</v>
+      </c>
+      <c r="C55">
+        <v>2016</v>
+      </c>
+      <c r="D55" t="s">
+        <v>84</v>
+      </c>
+      <c r="E55">
+        <v>24</v>
+      </c>
+      <c r="F55">
+        <v>2146</v>
+      </c>
+      <c r="G55">
+        <v>4</v>
+      </c>
+      <c r="H55">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56">
+        <v>913</v>
+      </c>
+      <c r="B56" t="s">
+        <v>52</v>
+      </c>
+      <c r="C56">
+        <v>2016</v>
+      </c>
+      <c r="D56" t="s">
+        <v>90</v>
+      </c>
+      <c r="F56">
+        <v>2333</v>
+      </c>
+      <c r="G56">
+        <v>4</v>
+      </c>
+      <c r="H56">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57">
+        <v>915</v>
+      </c>
+      <c r="B57" t="s">
+        <v>53</v>
+      </c>
+      <c r="C57">
+        <v>2017</v>
+      </c>
+      <c r="D57" t="s">
+        <v>74</v>
+      </c>
+      <c r="E57">
+        <v>51</v>
+      </c>
+      <c r="F57">
+        <v>961</v>
+      </c>
+      <c r="G57">
+        <v>4</v>
+      </c>
+      <c r="H57">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58">
+        <v>926</v>
+      </c>
+      <c r="B58" t="s">
+        <v>54</v>
+      </c>
+      <c r="C58">
+        <v>2017</v>
+      </c>
+      <c r="D58" t="s">
+        <v>91</v>
+      </c>
+      <c r="F58">
+        <v>259</v>
+      </c>
+      <c r="G58">
+        <v>5</v>
+      </c>
+      <c r="H58">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59">
+        <v>975</v>
+      </c>
+      <c r="B59" t="s">
+        <v>55</v>
+      </c>
+      <c r="C59">
+        <v>2017</v>
+      </c>
+      <c r="D59" t="s">
+        <v>84</v>
+      </c>
+      <c r="E59">
+        <v>25</v>
+      </c>
+      <c r="F59">
+        <v>2085</v>
+      </c>
+      <c r="G59">
+        <v>5</v>
+      </c>
+      <c r="H59">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60">
+        <v>992</v>
+      </c>
+      <c r="B60" t="s">
+        <v>56</v>
+      </c>
+      <c r="C60">
+        <v>2017</v>
+      </c>
+      <c r="D60" t="s">
+        <v>92</v>
+      </c>
+      <c r="F60">
+        <v>763</v>
+      </c>
+      <c r="G60">
+        <v>4</v>
+      </c>
+      <c r="H60">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61">
+        <v>1177</v>
+      </c>
+      <c r="B61" t="s">
         <v>57</v>
       </c>
-      <c r="E33">
-        <v>139</v>
-      </c>
-      <c r="G33">
-        <v>13</v>
-      </c>
-      <c r="H33">
-        <v>7</v>
+      <c r="C61">
+        <v>2019</v>
+      </c>
+      <c r="D61" t="s">
+        <v>93</v>
+      </c>
+      <c r="E61">
+        <v>29</v>
+      </c>
+      <c r="F61">
+        <v>2822</v>
+      </c>
+      <c r="G61">
+        <v>5</v>
+      </c>
+      <c r="H61">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62">
+        <v>1178</v>
+      </c>
+      <c r="B62" t="s">
+        <v>58</v>
+      </c>
+      <c r="C62">
+        <v>2019</v>
+      </c>
+      <c r="D62" t="s">
+        <v>94</v>
+      </c>
+      <c r="F62">
+        <v>722</v>
+      </c>
+      <c r="G62">
+        <v>2</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63">
+        <v>1311</v>
+      </c>
+      <c r="B63" t="s">
+        <v>59</v>
+      </c>
+      <c r="C63">
+        <v>2020</v>
+      </c>
+      <c r="D63" t="s">
+        <v>95</v>
+      </c>
+      <c r="F63">
+        <v>1366</v>
+      </c>
+      <c r="G63">
+        <v>2</v>
+      </c>
+      <c r="H63">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64">
+        <v>1337</v>
+      </c>
+      <c r="B64" t="s">
+        <v>60</v>
+      </c>
+      <c r="C64">
+        <v>2020</v>
+      </c>
+      <c r="D64" t="s">
+        <v>96</v>
+      </c>
+      <c r="E64">
+        <v>8</v>
+      </c>
+      <c r="F64">
+        <v>181340</v>
+      </c>
+      <c r="G64">
+        <v>2</v>
+      </c>
+      <c r="H64">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>